<commit_message>
테이블 수정: 몬스터, 레벨, wave, weapon level
</commit_message>
<xml_diff>
--- a/Table/TableAsset/TB_Level.xlsx
+++ b/Table/TableAsset/TB_Level.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -453,27 +453,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>level</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>required_exp</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>required_exp_gap</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>difficulty_multiplier</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -484,10 +484,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -503,10 +503,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="C3" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="D3" t="n">
         <v>1.1</v>
@@ -517,10 +517,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
       <c r="C4" t="n">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="D4" t="n">
         <v>1.2</v>
@@ -531,10 +531,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>180</v>
+        <v>63</v>
       </c>
       <c r="C5" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="D5" t="n">
         <v>1.3</v>
@@ -545,10 +545,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>250</v>
+        <v>98</v>
       </c>
       <c r="C6" t="n">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="D6" t="n">
         <v>1.5</v>
@@ -564,10 +564,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>330</v>
+        <v>143</v>
       </c>
       <c r="C7" t="n">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="D7" t="n">
         <v>1.6</v>
@@ -578,10 +578,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>420</v>
+        <v>203</v>
       </c>
       <c r="C8" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="D8" t="n">
         <v>1.8</v>
@@ -592,10 +592,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>520</v>
+        <v>283</v>
       </c>
       <c r="C9" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="D9" t="n">
         <v>2</v>
@@ -611,10 +611,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>630</v>
+        <v>383</v>
       </c>
       <c r="C10" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="D10" t="n">
         <v>2.2</v>
@@ -625,10 +625,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>750</v>
+        <v>513</v>
       </c>
       <c r="C11" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="D11" t="n">
         <v>2.5</v>
@@ -636,109 +636,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>최대 레벨</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>[컬럼명]</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>[타입]</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>[설명]</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>level</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>int (PK)</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>플레이어 레벨</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>required_exp</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>누적 필요 경험치</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>required_exp_gap</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>이전 레벨 대비 증가량</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>difficulty_multiplier</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>난이도 배율</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>비고</t>
         </is>
       </c>
     </row>

</xml_diff>